<commit_message>
Phantom details template updated.
</commit_message>
<xml_diff>
--- a/PhantomExtraction/PhantomDetails.xlsx
+++ b/PhantomExtraction/PhantomDetails.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leonardobertini/PycharmProjects/CoralMethodsPaper/PhantomExtraction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04F91829-0534-C94B-A248-A85585FA8485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A2C1AF4-F402-4148-89C2-30048517A8F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{F8590A82-7C93-424B-B265-32E5B91FD80B}"/>
   </bookViews>
@@ -735,7 +735,7 @@
         <v>0.90400000000000003</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -746,7 +746,7 @@
         <v>0.26</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -762,5 +762,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixing RGB to BGR colour codes for plotting diagnostic figures.
</commit_message>
<xml_diff>
--- a/PhantomExtraction/PhantomDetails.xlsx
+++ b/PhantomExtraction/PhantomDetails.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leonardobertini/PycharmProjects/CoralMethodsPaper/PhantomExtraction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A2C1AF4-F402-4148-89C2-30048517A8F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6977BD3-51D9-1D4F-B938-C3163F303F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{F8590A82-7C93-424B-B265-32E5B91FD80B}"/>
   </bookViews>
@@ -735,7 +735,7 @@
         <v>0.90400000000000003</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -746,7 +746,7 @@
         <v>0.26</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>